<commit_message>
Revised Aug 25, 2025
Updates the given solution to the business jet problem to one that meets the equality constraints exactly.
</commit_message>
<xml_diff>
--- a/Benchmarks/businessjet/bjet_solution.xlsx
+++ b/Benchmarks/businessjet/bjet_solution.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11028"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donaldjones/Desktop/GOMDO/Benchmarks/businessjet/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donaldjones/Documents/GOMDO/GOMDO_core_faster/Benchmarks/businessjet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E4C66D8-146E-A740-91B9-4E974271378C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1D5D96A-23E2-7F43-A395-E0DB3A6AD6B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5780" yWindow="500" windowWidth="27640" windowHeight="16940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-32320" yWindow="1600" windowWidth="27640" windowHeight="16940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Best Opt from Multistart" sheetId="3" r:id="rId1"/>
@@ -462,7 +462,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -470,6 +470,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -811,7 +812,7 @@
     <col min="2" max="2" width="12.1640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="6.1640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.6640625" customWidth="1"/>
     <col min="7" max="7" width="6.83203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.83203125" bestFit="1" customWidth="1"/>
@@ -897,13 +898,14 @@
       <c r="H1" s="2" t="s">
         <v>121</v>
       </c>
+      <c r="I1" s="2"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B2">
-        <v>4.8742978961727579E-2</v>
+        <v>4.8745439089062682E-2</v>
       </c>
       <c r="C2">
         <v>0.01</v>
@@ -915,9 +917,9 @@
         <v>41</v>
       </c>
       <c r="H2">
-        <v>32.635338666009197</v>
-      </c>
-      <c r="J2" t="s">
+        <v>32.636883060501297</v>
+      </c>
+      <c r="J2" s="3" t="s">
         <v>125</v>
       </c>
     </row>
@@ -938,7 +940,7 @@
         <v>42</v>
       </c>
       <c r="H3">
-        <v>-0.32407753234693149</v>
+        <v>-0.35579227374251299</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
@@ -958,7 +960,7 @@
         <v>43</v>
       </c>
       <c r="H4">
-        <v>-0.59195240741751931</v>
+        <v>-0.56363631467407582</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
@@ -978,7 +980,7 @@
         <v>44</v>
       </c>
       <c r="H5">
-        <v>-0.53822097218455345</v>
+        <v>-0.52773575383823812</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
@@ -998,7 +1000,7 @@
         <v>45</v>
       </c>
       <c r="H6">
-        <v>-0.16961525199483851</v>
+        <v>-0.20398953337757531</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
@@ -1006,7 +1008,7 @@
         <v>5</v>
       </c>
       <c r="B7">
-        <v>663.08194577304118</v>
+        <v>663.09960977857986</v>
       </c>
       <c r="C7">
         <v>200</v>
@@ -1018,7 +1020,7 @@
         <v>46</v>
       </c>
       <c r="H7">
-        <v>-0.77310537472221319</v>
+        <v>-0.6860760747600041</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
@@ -1026,7 +1028,7 @@
         <v>6</v>
       </c>
       <c r="B8">
-        <v>82.592832345430779</v>
+        <v>82.584686013242816</v>
       </c>
       <c r="C8">
         <v>50</v>
@@ -1038,7 +1040,7 @@
         <v>47</v>
       </c>
       <c r="H8">
-        <v>-0.27559840954261405</v>
+        <v>-0.33697292239213206</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
@@ -1058,7 +1060,7 @@
         <v>48</v>
       </c>
       <c r="H9">
-        <v>-1.3933982024820388</v>
+        <v>-0.91050886968803324</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
@@ -1066,7 +1068,7 @@
         <v>8</v>
       </c>
       <c r="B10">
-        <v>1.8423126270116177</v>
+        <v>1.8422232995108232</v>
       </c>
       <c r="C10">
         <v>0.1</v>
@@ -1078,7 +1080,7 @@
         <v>49</v>
       </c>
       <c r="H10">
-        <v>-1.2233030466833275</v>
+        <v>-0.87093234795641772</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
@@ -1086,7 +1088,7 @@
         <v>9</v>
       </c>
       <c r="B11">
-        <v>0.61161166635851638</v>
+        <v>0.61211484066182831</v>
       </c>
       <c r="C11">
         <v>0.1</v>
@@ -1098,7 +1100,7 @@
         <v>50</v>
       </c>
       <c r="H11">
-        <v>-1.5942875388154949</v>
+        <v>-0.93600686590281579</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
@@ -1106,7 +1108,7 @@
         <v>10</v>
       </c>
       <c r="B12">
-        <v>0.23558433799588621</v>
+        <v>0.23603343011249014</v>
       </c>
       <c r="C12">
         <v>0.1</v>
@@ -1118,7 +1120,7 @@
         <v>51</v>
       </c>
       <c r="H12">
-        <v>-0.8355659230396153</v>
+        <v>-0.7218490037473797</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
@@ -1126,7 +1128,7 @@
         <v>11</v>
       </c>
       <c r="B13">
-        <v>0.22231350105083961</v>
+        <v>0.22833896362009237</v>
       </c>
       <c r="C13">
         <v>0.1</v>
@@ -1138,7 +1140,7 @@
         <v>52</v>
       </c>
       <c r="H13">
-        <v>-0.69291150399603929</v>
+        <v>-0.63867355707812479</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
@@ -1146,7 +1148,7 @@
         <v>12</v>
       </c>
       <c r="B14">
-        <v>0.35416720080381375</v>
+        <v>0.34352357290655061</v>
       </c>
       <c r="C14">
         <v>0.1</v>
@@ -1158,7 +1160,7 @@
         <v>53</v>
       </c>
       <c r="H14">
-        <v>-0.78867515270400534</v>
+        <v>-0.69658466654794515</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
@@ -1178,7 +1180,7 @@
         <v>54</v>
       </c>
       <c r="H15">
-        <v>-1.170175067954915E-13</v>
+        <v>-6.668817498223234E-9</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
@@ -1186,7 +1188,7 @@
         <v>14</v>
       </c>
       <c r="B16">
-        <v>1.8423126270116179</v>
+        <v>1.842223296296853</v>
       </c>
       <c r="C16">
         <v>0.1</v>
@@ -1198,7 +1200,7 @@
         <v>55</v>
       </c>
       <c r="H16">
-        <v>-1.0302869668521453E-13</v>
+        <v>-1.0785071424823656E-7</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
@@ -1206,7 +1208,7 @@
         <v>15</v>
       </c>
       <c r="B17">
-        <v>0.61161163738239654</v>
+        <v>0.61206454553676803</v>
       </c>
       <c r="C17">
         <v>0.1</v>
@@ -1218,7 +1220,7 @@
         <v>56</v>
       </c>
       <c r="H17">
-        <v>-1.9995116673499069E-13</v>
+        <v>-9.3338877022364208E-3</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
@@ -1226,7 +1228,7 @@
         <v>16</v>
       </c>
       <c r="B18">
-        <v>0.2355843666211167</v>
+        <v>0.23662301012696965</v>
       </c>
       <c r="C18">
         <v>0.1</v>
@@ -1238,7 +1240,7 @@
         <v>57</v>
       </c>
       <c r="H18">
-        <v>-1.9991429476331057</v>
+        <v>-0.97480317484847245</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
@@ -1258,7 +1260,7 @@
         <v>58</v>
       </c>
       <c r="H19">
-        <v>-1.9988017736561488</v>
+        <v>-0.97478475224954719</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
@@ -1266,7 +1268,7 @@
         <v>18</v>
       </c>
       <c r="B20">
-        <v>1.8813582745741553</v>
+        <v>1.8807294859950179</v>
       </c>
       <c r="C20">
         <v>0.1</v>
@@ -1278,7 +1280,7 @@
         <v>59</v>
       </c>
       <c r="H20">
-        <v>-1.9972855476849785</v>
+        <v>-0.97423418684572916</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
@@ -1286,7 +1288,7 @@
         <v>19</v>
       </c>
       <c r="B21">
-        <v>0.94125267014980618</v>
+        <v>0.94519375199861744</v>
       </c>
       <c r="C21">
         <v>0.1</v>
@@ -1298,7 +1300,7 @@
         <v>60</v>
       </c>
       <c r="H21">
-        <v>-0.10849309625558123</v>
+        <v>-0.14235112686984774</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
@@ -1306,7 +1308,7 @@
         <v>20</v>
       </c>
       <c r="B22">
-        <v>0.29858358094233389</v>
+        <v>0.29953293078772381</v>
       </c>
       <c r="C22">
         <v>0.1</v>
@@ -1318,7 +1320,7 @@
         <v>61</v>
       </c>
       <c r="H22">
-        <v>-0.51249131930566216</v>
+        <v>-0.49884977898377569</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
@@ -1326,7 +1328,7 @@
         <v>21</v>
       </c>
       <c r="B23">
-        <v>0.3895839208848334</v>
+        <v>0.38759486337032961</v>
       </c>
       <c r="C23">
         <v>0.1</v>
@@ -1338,7 +1340,7 @@
         <v>62</v>
       </c>
       <c r="H23">
-        <v>-0.40674000225033424</v>
+        <v>-0.41651892056102424</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
@@ -1346,7 +1348,7 @@
         <v>22</v>
       </c>
       <c r="B24">
-        <v>0.11</v>
+        <v>0.11328593508579471</v>
       </c>
       <c r="C24">
         <v>0.1</v>
@@ -1358,7 +1360,7 @@
         <v>63</v>
       </c>
       <c r="H24">
-        <v>-1.0658141036401503E-14</v>
+        <v>-3.442279399290249E-2</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
@@ -1378,7 +1380,7 @@
         <v>64</v>
       </c>
       <c r="H25">
-        <v>-0.7717113123315068</v>
+        <v>-0.68520066215666198</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
@@ -1386,7 +1388,7 @@
         <v>24</v>
       </c>
       <c r="B26">
-        <v>1.8813583541851671</v>
+        <v>1.8808674458447467</v>
       </c>
       <c r="C26">
         <v>0.1</v>
@@ -1398,7 +1400,7 @@
         <v>65</v>
       </c>
       <c r="H26">
-        <v>-0.22509496067581225</v>
+        <v>-0.29285410697312619</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
@@ -1406,7 +1408,7 @@
         <v>25</v>
       </c>
       <c r="B27">
-        <v>0.94125255918029482</v>
+        <v>0.9429481609274083</v>
       </c>
       <c r="C27">
         <v>0.1</v>
@@ -1418,7 +1420,7 @@
         <v>66</v>
       </c>
       <c r="H27">
-        <v>-1.2237829504872111</v>
+        <v>-0.87593706374810221</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.2">
@@ -1438,7 +1440,7 @@
         <v>67</v>
       </c>
       <c r="H28">
-        <v>-1.2219089842926212</v>
+        <v>-0.87053284545230436</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.2">
@@ -1458,7 +1460,7 @@
         <v>68</v>
       </c>
       <c r="H29">
-        <v>-1.5437840899486932</v>
+        <v>-0.92965128469606084</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.2">
@@ -1478,7 +1480,7 @@
         <v>69</v>
       </c>
       <c r="H30">
-        <v>-1.1457501614131615E-13</v>
+        <v>-2.8169192074715577E-2</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
@@ -1498,7 +1500,7 @@
         <v>70</v>
       </c>
       <c r="H31">
-        <v>-0.47001748624831785</v>
+        <v>-0.46178710112715082</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
@@ -1506,7 +1508,7 @@
         <v>30</v>
       </c>
       <c r="B32">
-        <v>0.15625054394214274</v>
+        <v>0.15625054393685894</v>
       </c>
       <c r="C32">
         <v>0.1</v>
@@ -1518,7 +1520,7 @@
         <v>71</v>
       </c>
       <c r="H32">
-        <v>-0.3395449659485521</v>
+        <v>-0.35423653030703761</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
@@ -1526,7 +1528,7 @@
         <v>31</v>
       </c>
       <c r="B33">
-        <v>32635.338666009196</v>
+        <v>32636.883060501295</v>
       </c>
       <c r="C33">
         <v>5000</v>
@@ -1538,7 +1540,7 @@
         <v>72</v>
       </c>
       <c r="H33">
-        <v>-0.8355659230396153</v>
+        <v>-0.72184900359842064</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
@@ -1546,7 +1548,7 @@
         <v>32</v>
       </c>
       <c r="B34">
-        <v>6806.8361670204667</v>
+        <v>6807.2622632231751</v>
       </c>
       <c r="C34">
         <v>100</v>
@@ -1558,7 +1560,7 @@
         <v>73</v>
       </c>
       <c r="H34">
-        <v>-0.6929114897783335</v>
+        <v>-0.6386576215847195</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.2">
@@ -1566,7 +1568,7 @@
         <v>33</v>
       </c>
       <c r="B35">
-        <v>32635.338666009196</v>
+        <v>32636.883060501295</v>
       </c>
       <c r="C35">
         <v>5000</v>
@@ -1578,7 +1580,7 @@
         <v>74</v>
       </c>
       <c r="H35">
-        <v>-0.78867517795059072</v>
+        <v>-0.69687489214987519</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.2">
@@ -1586,7 +1588,7 @@
         <v>34</v>
       </c>
       <c r="B36">
-        <v>14.466940263529555</v>
+        <v>14.465988181269047</v>
       </c>
       <c r="C36">
         <v>0.2</v>
@@ -1598,7 +1600,7 @@
         <v>75</v>
       </c>
       <c r="H36">
-        <v>-1.9991429476331053</v>
+        <v>-0.97480317514243919</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.2">
@@ -1606,7 +1608,7 @@
         <v>35</v>
       </c>
       <c r="B37">
-        <v>0.78986205407680676</v>
+        <v>0.78990914353245756</v>
       </c>
       <c r="C37">
         <v>0.5</v>
@@ -1618,7 +1620,7 @@
         <v>76</v>
       </c>
       <c r="H37">
-        <v>-1.9988017736536592</v>
+        <v>-0.97478475619046534</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.2">
@@ -1626,7 +1628,7 @@
         <v>36</v>
       </c>
       <c r="B38">
-        <v>3990.7919210381178</v>
+        <v>3991.0298412060852</v>
       </c>
       <c r="C38">
         <v>1000</v>
@@ -1638,7 +1640,7 @@
         <v>77</v>
       </c>
       <c r="H38">
-        <v>-1.9972855476965901</v>
+        <v>-0.97423071869492595</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.2">
@@ -1646,7 +1648,7 @@
         <v>37</v>
       </c>
       <c r="B39">
-        <v>8152.9567203319248</v>
+        <v>8153.4501519585938</v>
       </c>
       <c r="C39">
         <v>5000</v>
@@ -1658,7 +1660,7 @@
         <v>78</v>
       </c>
       <c r="H39">
-        <v>-1.1768364061026659E-13</v>
+        <v>-7.5081674211219251E-10</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
@@ -1666,7 +1668,7 @@
         <v>38</v>
       </c>
       <c r="B40">
-        <v>8.0114443309606642</v>
+        <v>8.0113218532936177</v>
       </c>
       <c r="C40">
         <v>0.1</v>
@@ -1678,7 +1680,7 @@
         <v>79</v>
       </c>
       <c r="H40">
-        <v>4.2188474935755949E-14</v>
+        <v>-2.3678244143177096E-8</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">
@@ -1686,7 +1688,7 @@
         <v>39</v>
       </c>
       <c r="B41">
-        <v>0.92393308479045444</v>
+        <v>0.9239330847929248</v>
       </c>
       <c r="C41">
         <v>0.9</v>
@@ -1698,7 +1700,7 @@
         <v>80</v>
       </c>
       <c r="H41">
-        <v>-1.4832579608992091E-13</v>
+        <v>-9.4026802057858294E-3</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
@@ -1706,7 +1708,7 @@
         <v>40</v>
       </c>
       <c r="B42">
-        <v>17675.545778656808</v>
+        <v>17676.170645319526</v>
       </c>
       <c r="C42">
         <v>5000</v>
@@ -1718,7 +1720,7 @@
         <v>81</v>
       </c>
       <c r="H42">
-        <v>-0.43078208633933635</v>
+        <v>-0.4504073152368463</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.2">
@@ -1726,7 +1728,7 @@
         <v>82</v>
       </c>
       <c r="H43">
-        <v>-0.627813042735056</v>
+        <v>-0.59090646642400269</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">
@@ -1734,7 +1736,7 @@
         <v>83</v>
       </c>
       <c r="H44">
-        <v>-0.60163040780681243</v>
+        <v>-0.5760195448884764</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.2">
@@ -1742,7 +1744,7 @@
         <v>84</v>
       </c>
       <c r="H45">
-        <v>-0.99354333357583635</v>
+        <v>-0.79460452621774613</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.2">
@@ -1750,7 +1752,7 @@
         <v>85</v>
       </c>
       <c r="H46">
-        <v>-0.79165812282498871</v>
+        <v>-0.69814619569044867</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.2">
@@ -1758,7 +1760,7 @@
         <v>86</v>
       </c>
       <c r="H47">
-        <v>-0.82220035368585653</v>
+        <v>-0.71445364970665948</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.2">
@@ -1766,7 +1768,7 @@
         <v>87</v>
       </c>
       <c r="H48">
-        <v>-22.872076565536364</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="49" spans="7:8" x14ac:dyDescent="0.2">
@@ -1774,7 +1776,7 @@
         <v>88</v>
       </c>
       <c r="H49">
-        <v>-0.66398602454034483</v>
+        <v>-0.61929876059216493</v>
       </c>
     </row>
     <row r="50" spans="7:8" x14ac:dyDescent="0.2">
@@ -1782,7 +1784,7 @@
         <v>89</v>
       </c>
       <c r="H50">
-        <v>-0.74328667581826169</v>
+        <v>-0.67039609900945196</v>
       </c>
     </row>
     <row r="51" spans="7:8" x14ac:dyDescent="0.2">
@@ -1790,7 +1792,7 @@
         <v>90</v>
       </c>
       <c r="H51">
-        <v>-0.19554294757343571</v>
+        <v>-0.18837540531673314</v>
       </c>
     </row>
     <row r="52" spans="7:8" x14ac:dyDescent="0.2">
@@ -1798,7 +1800,7 @@
         <v>91</v>
       </c>
       <c r="H52">
-        <v>-1.8022250358740166E-12</v>
+        <v>-3.0003917140208336E-2</v>
       </c>
     </row>
     <row r="53" spans="7:8" x14ac:dyDescent="0.2">
@@ -1806,7 +1808,7 @@
         <v>92</v>
       </c>
       <c r="H53">
-        <v>0</v>
+        <v>-3.4690150500446326E-2</v>
       </c>
     </row>
     <row r="54" spans="7:8" x14ac:dyDescent="0.2">
@@ -1814,7 +1816,7 @@
         <v>93</v>
       </c>
       <c r="H54">
-        <v>-22.872076565536361</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="55" spans="7:8" x14ac:dyDescent="0.2">
@@ -1822,7 +1824,7 @@
         <v>94</v>
       </c>
       <c r="H55">
-        <v>-0.66398605569090963</v>
+        <v>-0.61933512348347042</v>
       </c>
     </row>
     <row r="56" spans="7:8" x14ac:dyDescent="0.2">
@@ -1830,7 +1832,7 @@
         <v>95</v>
       </c>
       <c r="H56">
-        <v>-0.74328661278262809</v>
+        <v>-0.66962458531497493</v>
       </c>
     </row>
     <row r="57" spans="7:8" x14ac:dyDescent="0.2">
@@ -1838,7 +1840,7 @@
         <v>96</v>
       </c>
       <c r="H57">
-        <v>-1.6759224676530686</v>
+        <v>-0.94779405669106809</v>
       </c>
     </row>
     <row r="58" spans="7:8" x14ac:dyDescent="0.2">
@@ -1846,7 +1848,7 @@
         <v>97</v>
       </c>
       <c r="H58">
-        <v>-1.4080475925824807</v>
+        <v>-0.91271356219975475</v>
       </c>
     </row>
     <row r="59" spans="7:8" x14ac:dyDescent="0.2">
@@ -1854,7 +1856,7 @@
         <v>98</v>
       </c>
       <c r="H59">
-        <v>-1.4617790278154466</v>
+        <v>-0.92086480796254144</v>
       </c>
     </row>
     <row r="60" spans="7:8" x14ac:dyDescent="0.2">
@@ -1862,7 +1864,7 @@
         <v>99</v>
       </c>
       <c r="H60">
-        <v>-1.1644340769603847</v>
+        <v>-0.85385003085159583</v>
       </c>
     </row>
     <row r="61" spans="7:8" x14ac:dyDescent="0.2">
@@ -1870,7 +1872,7 @@
         <v>100</v>
       </c>
       <c r="H61">
-        <v>-1.3070884960039608</v>
+        <v>-0.89079397597470511</v>
       </c>
     </row>
     <row r="62" spans="7:8" x14ac:dyDescent="0.2">
@@ -1878,7 +1880,7 @@
         <v>101</v>
       </c>
       <c r="H62">
-        <v>-1.2113248472959945</v>
+        <v>-0.86704562592448275</v>
       </c>
     </row>
     <row r="63" spans="7:8" x14ac:dyDescent="0.2">
@@ -1886,7 +1888,7 @@
         <v>102</v>
       </c>
       <c r="H63">
-        <v>-1.8915069037444188</v>
+        <v>-0.96664010537486322</v>
       </c>
     </row>
     <row r="64" spans="7:8" x14ac:dyDescent="0.2">
@@ -1894,7 +1896,7 @@
         <v>103</v>
       </c>
       <c r="H64">
-        <v>-1.4875086806943378</v>
+        <v>-0.9266170336382229</v>
       </c>
     </row>
     <row r="65" spans="7:8" x14ac:dyDescent="0.2">
@@ -1902,7 +1904,7 @@
         <v>104</v>
       </c>
       <c r="H65">
-        <v>-1.5932599977496658</v>
+        <v>-0.94001932567957014</v>
       </c>
     </row>
     <row r="66" spans="7:8" x14ac:dyDescent="0.2">
@@ -1910,7 +1912,7 @@
         <v>105</v>
       </c>
       <c r="H66">
-        <v>-1.9999999999998854</v>
+        <v>-0.97341105132476868</v>
       </c>
     </row>
     <row r="67" spans="7:8" x14ac:dyDescent="0.2">
@@ -1918,7 +1920,7 @@
         <v>106</v>
       </c>
       <c r="H67">
-        <v>-1.529982513751682</v>
+        <v>-0.93313454699886755</v>
       </c>
     </row>
     <row r="68" spans="7:8" x14ac:dyDescent="0.2">
@@ -1926,7 +1928,7 @@
         <v>107</v>
       </c>
       <c r="H68">
-        <v>-1.6604550340514479</v>
+        <v>-0.94797476354392363</v>
       </c>
     </row>
     <row r="69" spans="7:8" x14ac:dyDescent="0.2">
@@ -1934,7 +1936,7 @@
         <v>108</v>
       </c>
       <c r="H69">
-        <v>-1.1644340769603847</v>
+        <v>-0.85385003093586431</v>
       </c>
     </row>
     <row r="70" spans="7:8" x14ac:dyDescent="0.2">
@@ -1942,7 +1944,7 @@
         <v>109</v>
       </c>
       <c r="H70">
-        <v>-1.3070885102216665</v>
+        <v>-0.89079953304963111</v>
       </c>
     </row>
     <row r="71" spans="7:8" x14ac:dyDescent="0.2">
@@ -1950,7 +1952,7 @@
         <v>110</v>
       </c>
       <c r="H71">
-        <v>-1.2113248220494093</v>
+        <v>-0.86690555008008796</v>
       </c>
     </row>
     <row r="72" spans="7:8" x14ac:dyDescent="0.2">
@@ -1958,7 +1960,7 @@
         <v>111</v>
       </c>
       <c r="H72">
-        <v>-1.5692179136606637</v>
+        <v>-0.93496721764945545</v>
       </c>
     </row>
     <row r="73" spans="7:8" x14ac:dyDescent="0.2">
@@ -1966,7 +1968,7 @@
         <v>112</v>
       </c>
       <c r="H73">
-        <v>-1.3721869572649439</v>
+        <v>-0.90562247496558612</v>
       </c>
     </row>
     <row r="74" spans="7:8" x14ac:dyDescent="0.2">
@@ -1974,7 +1976,7 @@
         <v>113</v>
       </c>
       <c r="H74">
-        <v>-1.3983695921931876</v>
+        <v>-0.90960011457581214</v>
       </c>
     </row>
     <row r="75" spans="7:8" x14ac:dyDescent="0.2">
@@ -1982,7 +1984,7 @@
         <v>114</v>
       </c>
       <c r="H75">
-        <v>-9.5480076502808875E-2</v>
+        <v>-0.10376923139278582</v>
       </c>
     </row>
     <row r="76" spans="7:8" x14ac:dyDescent="0.2">
@@ -1990,7 +1992,7 @@
         <v>115</v>
       </c>
       <c r="H76">
-        <v>-0.25115129070802278</v>
+        <v>-0.26731883402098278</v>
       </c>
     </row>
     <row r="77" spans="7:8" x14ac:dyDescent="0.2">
@@ -1998,7 +2000,7 @@
         <v>116</v>
       </c>
       <c r="H77">
-        <v>-0.22911837601664575</v>
+        <v>-0.24485859004455846</v>
       </c>
     </row>
     <row r="78" spans="7:8" x14ac:dyDescent="0.2">
@@ -2006,7 +2008,7 @@
         <v>117</v>
       </c>
       <c r="H78">
-        <v>-0.12905497488251505</v>
+        <v>-0.1398561561354702</v>
       </c>
     </row>
     <row r="79" spans="7:8" x14ac:dyDescent="0.2">
@@ -2014,7 +2016,7 @@
         <v>118</v>
       </c>
       <c r="H79">
-        <v>0</v>
+        <v>-3.6888270216195451E-11</v>
       </c>
     </row>
     <row r="80" spans="7:8" x14ac:dyDescent="0.2">
@@ -2022,11 +2024,12 @@
         <v>119</v>
       </c>
       <c r="H80">
-        <v>1.1102230246251565E-16</v>
+        <v>-3.1146747403454356E-9</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>